<commit_message>
- rearrangement of files and classes to support clarity and extensibility - use excel sheet to define farms (farms.xlsx)
</commit_message>
<xml_diff>
--- a/InputData/farms.xlsx
+++ b/InputData/farms.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="63">
   <si>
     <t xml:space="preserve">farm_id</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t xml:space="preserve">pasture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">num_infected</t>
   </si>
   <si>
     <t xml:space="preserve">F1</t>
@@ -357,7 +360,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1048576"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="11.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.85"/>
@@ -368,7 +371,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="9" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" s="6" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -394,13 +398,16 @@
       <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
+      <c r="I1" s="6" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>75</v>
@@ -412,21 +419,24 @@
         <v>30</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>35</v>
@@ -438,21 +448,24 @@
         <v>30</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>135</v>
@@ -464,21 +477,24 @@
         <v>14</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>40</v>
@@ -490,21 +506,24 @@
         <v>14</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>125</v>
@@ -516,21 +535,24 @@
         <v>14</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>110</v>
@@ -542,21 +564,24 @@
         <v>14</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>100</v>
@@ -568,21 +593,24 @@
         <v>14</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>90</v>
@@ -594,21 +622,24 @@
         <v>14</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>45</v>
@@ -620,21 +651,24 @@
         <v>14</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>120</v>
@@ -646,21 +680,24 @@
         <v>14</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>50</v>
@@ -672,21 +709,24 @@
         <v>30</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>25</v>
@@ -698,21 +738,24 @@
         <v>90</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>50</v>
@@ -724,21 +767,24 @@
         <v>90</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="I14" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>80</v>
@@ -750,21 +796,24 @@
         <v>14</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="I15" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>100</v>
@@ -776,21 +825,24 @@
         <v>90</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="I16" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>330</v>
@@ -802,21 +854,24 @@
         <v>14</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="I17" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>55</v>
@@ -828,21 +883,24 @@
         <v>14</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="I18" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>90</v>
@@ -854,21 +912,24 @@
         <v>90</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>25</v>
@@ -880,17 +941,22 @@
         <v>14</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="21" s="6" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>62</v>
+      </c>
+      <c r="I20" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" s="6" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>

</xml_diff>

<commit_message>
Added infecting community and stopping the model when there is community spillover.
</commit_message>
<xml_diff>
--- a/InputData/farms.xlsx
+++ b/InputData/farms.xlsx
@@ -486,7 +486,7 @@
         <v>19</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -544,7 +544,7 @@
         <v>25</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -602,7 +602,7 @@
         <v>25</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -660,7 +660,7 @@
         <v>12</v>
       </c>
       <c r="I10" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -718,7 +718,7 @@
         <v>39</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -776,7 +776,7 @@
         <v>19</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -863,7 +863,7 @@
         <v>55</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -950,7 +950,7 @@
         <v>62</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" s="6" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Tracking the infection network and visualising it.   - drawing the network is not quite correct yet.
</commit_message>
<xml_diff>
--- a/InputData/farms.xlsx
+++ b/InputData/farms.xlsx
@@ -428,7 +428,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -486,7 +486,7 @@
         <v>19</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -544,7 +544,7 @@
         <v>25</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -602,7 +602,7 @@
         <v>25</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -718,7 +718,7 @@
         <v>39</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -776,7 +776,7 @@
         <v>19</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -863,7 +863,7 @@
         <v>55</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -950,7 +950,7 @@
         <v>62</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" s="6" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Farm service clinicians only start trips at the beginning and middle of the day.
</commit_message>
<xml_diff>
--- a/InputData/farms.xlsx
+++ b/InputData/farms.xlsx
@@ -23,15 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
   <si>
     <t xml:space="preserve">farm_id</t>
   </si>
   <si>
     <t xml:space="preserve">herd_size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">visit_num_people</t>
   </si>
   <si>
     <t xml:space="preserve">visit_frequency_days</t>
@@ -360,19 +357,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="11.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ22"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="2" min="2" style="1" width="20.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.51"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="9" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" s="6" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -386,7 +382,7 @@
       <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="5" t="s">
@@ -395,28 +391,26 @@
       <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>7</v>
-      </c>
+      <c r="AMJ1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>75</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="n">
         <v>30</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -424,260 +418,233 @@
       <c r="G2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="1" t="n">
+      <c r="H2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>35</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" s="1" t="n">
         <v>30</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="1" t="n">
+      <c r="H3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>135</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H4" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>40</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="1" t="n">
+      <c r="H5" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>125</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="H6" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>110</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="H7" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>100</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I8" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="H8" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>90</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="H9" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>45</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="H10" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>120</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>10</v>
@@ -685,283 +652,252 @@
       <c r="G11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I11" s="1" t="n">
+      <c r="H11" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>50</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E12" s="1" t="n">
         <v>30</v>
       </c>
+      <c r="E12" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="F12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I12" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="H12" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>25</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" s="1" t="n">
         <v>90</v>
       </c>
+      <c r="E13" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="F13" s="1" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I13" s="1" t="n">
+      <c r="H13" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>50</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" s="1" t="n">
         <v>90</v>
       </c>
+      <c r="E14" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F14" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="H14" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>80</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E15" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I15" s="1" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>100</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" s="1" t="n">
         <v>90</v>
       </c>
+      <c r="E16" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F16" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I16" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="H16" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>330</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E17" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="F17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="I17" s="1" t="n">
+      <c r="H17" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>55</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I18" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="H18" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>90</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E19" s="1" t="n">
         <v>90</v>
       </c>
+      <c r="E19" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="F19" s="1" t="s">
         <v>10</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I19" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="H19" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>25</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" s="1" t="n">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I20" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="H20" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21" s="6" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I21" s="1"/>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H21" s="1"/>
+      <c r="AMJ21" s="0"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.2" right="0.7" top="0.5" bottom="0.5" header="0.3" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Truck now infects/infected by environment of farm and hospital truck bay. (as well as any people that go in the truck)
</commit_message>
<xml_diff>
--- a/InputData/farms.xlsx
+++ b/InputData/farms.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="61">
   <si>
     <t xml:space="preserve">farm_id</t>
   </si>
@@ -41,9 +41,6 @@
   </si>
   <si>
     <t xml:space="preserve">pasture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">num_infected</t>
   </si>
   <si>
     <t xml:space="preserve">F1</t>
@@ -367,8 +364,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.51"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="9" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1022" min="8" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" s="6" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -391,17 +387,15 @@
       <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>6</v>
-      </c>
+      <c r="AMI1" s="0"/>
       <c r="AMJ1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>75</v>
@@ -410,24 +404,21 @@
         <v>30</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>35</v>
@@ -436,24 +427,21 @@
         <v>30</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>135</v>
@@ -462,24 +450,21 @@
         <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>40</v>
@@ -488,24 +473,21 @@
         <v>14</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="1" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>125</v>
@@ -514,24 +496,21 @@
         <v>14</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="1" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>110</v>
@@ -540,24 +519,21 @@
         <v>14</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H7" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>100</v>
@@ -566,24 +542,21 @@
         <v>14</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="1" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>90</v>
@@ -592,24 +565,21 @@
         <v>14</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" s="1" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>45</v>
@@ -618,24 +588,21 @@
         <v>14</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>120</v>
@@ -644,24 +611,21 @@
         <v>14</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H11" s="1" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>50</v>
@@ -670,24 +634,21 @@
         <v>30</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="1" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>25</v>
@@ -696,24 +657,21 @@
         <v>90</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="H13" s="1" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>50</v>
@@ -722,24 +680,21 @@
         <v>90</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H14" s="1" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>80</v>
@@ -748,24 +703,21 @@
         <v>14</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H15" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>100</v>
@@ -774,24 +726,21 @@
         <v>90</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="H16" s="1" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>330</v>
@@ -800,24 +749,21 @@
         <v>14</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H17" s="1" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>55</v>
@@ -826,24 +772,21 @@
         <v>14</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H18" s="1" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>90</v>
@@ -852,24 +795,21 @@
         <v>90</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H19" s="1" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>25</v>
@@ -878,20 +818,17 @@
         <v>14</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H20" s="1" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" s="6" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H21" s="1"/>
+      <c r="AMI21" s="0"/>
       <c r="AMJ21" s="0"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>